<commit_message>
updated test data to align with date implementation update. Reran validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000097/negative/01/data/unit-test-coreid-CG0218-negative.xlsx
+++ b/rules/CORE-000097/negative/01/data/unit-test-coreid-CG0218-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-000097\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA808EDE-BE2B-4686-A260-BDF89995D387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89E8B7C-CF54-470F-AE12-8DFE629E9449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8385" yWindow="735" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="109">
   <si>
     <t>Product</t>
   </si>
@@ -324,9 +324,6 @@
     <t>2024-05-23</t>
   </si>
   <si>
-    <t>2024-06-01</t>
-  </si>
-  <si>
     <t>2024-06-02</t>
   </si>
   <si>
@@ -364,6 +361,9 @@
   </si>
   <si>
     <t>FOLLOW-UP5</t>
+  </si>
+  <si>
+    <t>2024-06-01T07:59</t>
   </si>
 </sst>
 </file>
@@ -474,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -518,6 +518,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -880,7 +883,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
@@ -919,16 +922,16 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -939,10 +942,10 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
@@ -959,16 +962,16 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
         <v>54</v>
       </c>
       <c r="F4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -979,13 +982,13 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
         <v>106</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5" t="s">
-        <v>107</v>
       </c>
       <c r="F5" t="s">
         <v>74</v>
@@ -999,7 +1002,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D6">
         <v>6</v>
@@ -1019,7 +1022,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D7">
         <v>6</v>
@@ -1039,16 +1042,16 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1059,16 +1062,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s">
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>104</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1079,16 +1082,16 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1099,13 +1102,13 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11" t="s">
         <v>106</v>
-      </c>
-      <c r="D11">
-        <v>6</v>
-      </c>
-      <c r="E11" t="s">
-        <v>107</v>
       </c>
       <c r="F11" t="s">
         <v>74</v>
@@ -1119,7 +1122,7 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12">
         <v>6</v>
@@ -1139,7 +1142,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D13">
         <v>6</v>
@@ -1159,16 +1162,16 @@
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D14">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1179,16 +1182,16 @@
         <v>8</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D15">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
         <v>23</v>
       </c>
       <c r="F15" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1199,16 +1202,16 @@
         <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D16">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
         <v>54</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1219,16 +1222,16 @@
         <v>6</v>
       </c>
       <c r="C17" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17">
+        <v>6</v>
+      </c>
+      <c r="E17" t="s">
         <v>106</v>
       </c>
-      <c r="D17">
-        <v>8</v>
-      </c>
-      <c r="E17" t="s">
-        <v>107</v>
-      </c>
       <c r="F17" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1239,16 +1242,16 @@
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E18" t="s">
         <v>24</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1259,16 +1262,16 @@
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E19" t="s">
         <v>25</v>
       </c>
       <c r="F19" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1279,16 +1282,16 @@
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D20">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
       </c>
       <c r="F20" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1299,16 +1302,16 @@
         <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D21">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
         <v>23</v>
       </c>
       <c r="F21" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1319,16 +1322,16 @@
         <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D22">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
         <v>54</v>
       </c>
       <c r="F22" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1339,13 +1342,13 @@
         <v>6</v>
       </c>
       <c r="C23" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23">
+        <v>8</v>
+      </c>
+      <c r="E23" t="s">
         <v>106</v>
-      </c>
-      <c r="D23">
-        <v>8</v>
-      </c>
-      <c r="E23" t="s">
-        <v>107</v>
       </c>
       <c r="F23" t="s">
         <v>46</v>
@@ -1359,7 +1362,7 @@
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D24">
         <v>8</v>
@@ -1379,7 +1382,7 @@
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D25">
         <v>8</v>
@@ -1399,16 +1402,16 @@
         <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D26">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E26" t="s">
         <v>53</v>
       </c>
       <c r="F26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1419,16 +1422,16 @@
         <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D27">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E27" t="s">
         <v>23</v>
       </c>
       <c r="F27" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1439,16 +1442,16 @@
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D28">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E28" t="s">
         <v>54</v>
       </c>
       <c r="F28" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1459,16 +1462,16 @@
         <v>6</v>
       </c>
       <c r="C29" t="s">
+        <v>105</v>
+      </c>
+      <c r="D29">
+        <v>8</v>
+      </c>
+      <c r="E29" t="s">
         <v>106</v>
       </c>
-      <c r="D29">
-        <v>9</v>
-      </c>
-      <c r="E29" t="s">
-        <v>107</v>
-      </c>
       <c r="F29" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1479,16 +1482,16 @@
         <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D30">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" t="s">
         <v>24</v>
       </c>
       <c r="F30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1499,16 +1502,16 @@
         <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D31">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31" t="s">
         <v>25</v>
       </c>
       <c r="F31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1519,16 +1522,16 @@
         <v>8</v>
       </c>
       <c r="C32" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D32">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
       </c>
       <c r="F32" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1539,16 +1542,16 @@
         <v>8</v>
       </c>
       <c r="C33" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33" t="s">
         <v>23</v>
       </c>
       <c r="F33" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1559,16 +1562,16 @@
         <v>8</v>
       </c>
       <c r="C34" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D34">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E34" t="s">
         <v>54</v>
       </c>
       <c r="F34" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1579,13 +1582,13 @@
         <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D35">
         <v>9</v>
       </c>
       <c r="E35" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F35" t="s">
         <v>74</v>
@@ -1599,7 +1602,7 @@
         <v>6</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D36">
         <v>9</v>
@@ -1619,7 +1622,7 @@
         <v>6</v>
       </c>
       <c r="C37" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D37">
         <v>9</v>
@@ -1639,16 +1642,16 @@
         <v>8</v>
       </c>
       <c r="C38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D38">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E38" t="s">
         <v>53</v>
       </c>
       <c r="F38" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1659,16 +1662,16 @@
         <v>8</v>
       </c>
       <c r="C39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D39">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E39" t="s">
         <v>23</v>
       </c>
       <c r="F39" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1679,16 +1682,16 @@
         <v>8</v>
       </c>
       <c r="C40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D40">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E40" t="s">
         <v>54</v>
       </c>
       <c r="F40" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1699,16 +1702,16 @@
         <v>6</v>
       </c>
       <c r="C41" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41">
+        <v>9</v>
+      </c>
+      <c r="E41" t="s">
         <v>106</v>
       </c>
-      <c r="D41">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s">
-        <v>107</v>
-      </c>
       <c r="F41" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1719,16 +1722,16 @@
         <v>6</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D42">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E42" t="s">
         <v>24</v>
       </c>
       <c r="F42" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1739,15 +1742,135 @@
         <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D43">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E43" t="s">
         <v>25</v>
       </c>
       <c r="F43" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>8</v>
+      </c>
+      <c r="B44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44">
+        <v>21</v>
+      </c>
+      <c r="E44" t="s">
+        <v>53</v>
+      </c>
+      <c r="F44" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>8</v>
+      </c>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>105</v>
+      </c>
+      <c r="D45">
+        <v>21</v>
+      </c>
+      <c r="E45" t="s">
+        <v>23</v>
+      </c>
+      <c r="F45" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>8</v>
+      </c>
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>105</v>
+      </c>
+      <c r="D46">
+        <v>21</v>
+      </c>
+      <c r="E46" t="s">
+        <v>54</v>
+      </c>
+      <c r="F46" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>8</v>
+      </c>
+      <c r="B47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" t="s">
+        <v>105</v>
+      </c>
+      <c r="D47">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
+        <v>106</v>
+      </c>
+      <c r="F47" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>8</v>
+      </c>
+      <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" t="s">
+        <v>105</v>
+      </c>
+      <c r="D48">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s">
+        <v>24</v>
+      </c>
+      <c r="F48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>8</v>
+      </c>
+      <c r="B49" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>25</v>
+      </c>
+      <c r="F49" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2024,13 +2147,13 @@
       <c r="G7" s="5">
         <v>3</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="17" t="s">
         <v>78</v>
       </c>
       <c r="K7" s="5">
@@ -2284,7 +2407,7 @@
     <col min="4" max="4" width="22.85546875" customWidth="1"/>
     <col min="5" max="5" width="17.5703125" customWidth="1"/>
     <col min="6" max="6" width="33" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" customWidth="1"/>
     <col min="9" max="9" width="12.140625" customWidth="1"/>
     <col min="11" max="11" width="11.7109375" customWidth="1"/>
@@ -2493,13 +2616,13 @@
       <c r="D6" s="7">
         <v>10101</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="14" t="s">
         <v>89</v>
       </c>
       <c r="H6" s="9" t="s">
@@ -2725,13 +2848,13 @@
         <v>51</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G12" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>96</v>
       </c>
       <c r="I12" s="5">
         <v>200</v>
@@ -2804,10 +2927,10 @@
         <v>51</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I14" s="5">
         <v>-1</v>
@@ -2842,10 +2965,10 @@
         <v>74</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I15" s="5">
         <v>2</v>
@@ -2880,10 +3003,10 @@
         <v>74</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I16" s="5">
         <v>8</v>
@@ -2918,10 +3041,10 @@
         <v>74</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I17" s="5">
         <v>8</v>
@@ -2953,13 +3076,13 @@
         <v>72</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I18" s="5">
         <v>15</v>
@@ -2994,10 +3117,10 @@
         <v>74</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I19" s="5">
         <v>16</v>
@@ -3032,10 +3155,10 @@
         <v>51</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I20" s="5">
         <v>200</v>
@@ -3067,7 +3190,7 @@
         <v>46</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>89</v>

</xml_diff>